<commit_message>
Fix dry mass and electricity units in hydrogen tank inventories
Normalize the HDPE and aluminium recipes to the listed dry material totals in Evangelisti et al. (2017), retaining processing services separately. Convert source manufacturing energy from MJ to kWh and document the ambiguous published mass boundary in dataset and exchange comments.

Include the workbook content in the supplementary-inventory cache key. Verify mass and energy after Excel import on both Brightway stacks, migrations to ecoinvent 3.9 through 3.12, and cache invalidation. Preserve all other workbook activity blocks.
</commit_message>
<xml_diff>
--- a/premise/data/additional_inventories/lci-trucks.xlsx
+++ b/premise/data/additional_inventories/lci-trucks.xlsx
@@ -2082,7 +2082,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:I5092"/>
+  <dimension ref="A1:J5092"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="26.1640625" customWidth="1"/>
@@ -2627,23 +2627,27 @@
       <c r="A41" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="B41" s="5" t="s">
-        <v>28</v>
+      <c r="B41" s="5" t="inlineStr">
+        <is>
+          <t>Fuel tank, compressed hydrogen gas, 700bar, with HDPE liner</t>
+        </is>
       </c>
     </row>
     <row r="42" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A42" t="s">
         <v>2</v>
       </c>
-      <c r="B42" t="s">
-        <v>281</v>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>RER</t>
+        </is>
       </c>
     </row>
     <row r="43" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A43" t="s">
         <v>3</v>
       </c>
-      <c r="B43">
+      <c r="B43" t="n">
         <v>1</v>
       </c>
     </row>
@@ -2651,48 +2655,60 @@
       <c r="A44" t="s">
         <v>4</v>
       </c>
-      <c r="B44" t="s">
-        <v>291</v>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>Hydrogen tank</t>
+        </is>
       </c>
     </row>
     <row r="45" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A45" t="s">
         <v>5</v>
       </c>
-      <c r="B45" t="s">
-        <v>283</v>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>process</t>
+        </is>
       </c>
     </row>
     <row r="46" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A46" t="s">
         <v>6</v>
       </c>
-      <c r="B46" t="s">
-        <v>284</v>
+      <c r="B46" t="inlineStr">
+        <is>
+          <t>kilogram</t>
+        </is>
       </c>
     </row>
     <row r="47" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A47" t="s">
         <v>7</v>
       </c>
-      <c r="B47" t="s">
-        <v>285</v>
+      <c r="B47" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
       </c>
     </row>
     <row r="48" spans="1:7" x14ac:dyDescent="0.2">
       <c r="A48" t="s">
         <v>8</v>
       </c>
-      <c r="B48" t="s">
-        <v>292</v>
+      <c r="B48" t="inlineStr">
+        <is>
+          <t>Evangelisti et al. 2017, doi: 10.1016/j.jclepro.2016.11.159</t>
+        </is>
       </c>
     </row>
     <row r="49" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A49" t="s">
         <v>9</v>
       </c>
-      <c r="B49" t="s">
-        <v>293</v>
+      <c r="B49" t="inlineStr">
+        <is>
+          <t>700-bar hydrogen tank with HDPE (Type IV) liner. Reference output: 1 kg dry tank assembly including tank balance of plant, excluding stored hydrogen. Source listed dry materials total 87.71 kg per assembly.</t>
+        </is>
       </c>
     </row>
     <row r="50" spans="1:9" x14ac:dyDescent="0.2">
@@ -2704,18 +2720,25 @@
       <c r="A51" t="s">
         <v>11</v>
       </c>
+      <c r="B51" t="inlineStr">
+        <is>
+          <t>Dry-mass correction, 2026-10-10. Evangelisti et al. (2017), doi:10.1016/j.jclepro.2016.11.159, supplementary Hydrogen tank (Scenario S16). Supplement: https://ars.els-cdn.com/content/image/1-s2.0-S0959652616320212-mmc1.docx. SHA256: ca9470c504f61ef58e2e5cc3cad8c06d6cecf17073074ac2ce19dca3678ac49d. Normalize all listed material and processing quantities by 87.71 kg of listed dry materials, not the legacy 119 kg denominator. The main text, scenario labels and supplementary output masses are inconsistent. The difference between nominal output and listed material mass is approximately stored hydrogen, but this interpretation is not explicit in the paper. Dry mass is an explicit modelling boundary, not an assumed missing material. Processing services do not add material mass. Preserve published material ratios and existing supplier proxies, including AlLi for aluminium; these are not validated as current vehicle specifications. Electricity is published in MJ: divide by 3.6 to obtain kWh.</t>
+        </is>
+      </c>
     </row>
     <row r="52" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A52" s="5" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="53" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="53" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A53" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="B53" s="5" t="s">
-        <v>288</v>
+      <c r="B53" s="5" t="inlineStr">
+        <is>
+          <t>amount</t>
+        </is>
       </c>
       <c r="C53" s="5" t="s">
         <v>417</v>
@@ -2738,13 +2761,18 @@
       <c r="I53" s="5" t="s">
         <v>486</v>
       </c>
-    </row>
-    <row r="54" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J53" t="inlineStr">
+        <is>
+          <t>comment</t>
+        </is>
+      </c>
+    </row>
+    <row r="54" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A54" t="s">
         <v>15</v>
       </c>
-      <c r="B54">
-        <v>0.108151261</v>
+      <c r="B54" t="n">
+        <v>0.04075932048797173</v>
       </c>
       <c r="C54" t="s">
         <v>418</v>
@@ -2764,13 +2792,18 @@
       <c r="I54" t="s">
         <v>544</v>
       </c>
-    </row>
-    <row r="55" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J54" t="inlineStr">
+        <is>
+          <t>12.87 MJ / 3.6 MJ/kWh / 87.71 kg dry assembly = 0.040759320488 kWh/kg. Evangelisti et al. (2017), supplementary Hydrogen tank (Scenario S16). Preserve existing supplier proxy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="55" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A55" t="s">
         <v>21</v>
       </c>
-      <c r="B55">
-        <v>8.9411765000000004E-2</v>
+      <c r="B55" t="n">
+        <v>0.1213088587390263</v>
       </c>
       <c r="C55" t="s">
         <v>418</v>
@@ -2790,13 +2823,18 @@
       <c r="I55" t="s">
         <v>487</v>
       </c>
-    </row>
-    <row r="56" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J55" t="inlineStr">
+        <is>
+          <t>(10.64) kg / 87.71 kg dry assembly = 0.121308858739 kg/kg. Processing service; excluded from material mass balance. Evangelisti et al. (2017), supplementary Hydrogen tank (Scenario S16). Preserve existing supplier proxy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="56" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A56" t="s">
         <v>23</v>
       </c>
-      <c r="B56">
-        <v>8.6218486999999996E-2</v>
+      <c r="B56" t="n">
+        <v>0.1169763994983468</v>
       </c>
       <c r="C56" t="s">
         <v>418</v>
@@ -2816,13 +2854,18 @@
       <c r="I56" t="s">
         <v>488</v>
       </c>
-    </row>
-    <row r="57" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J56" t="inlineStr">
+        <is>
+          <t>(10.26) kg / 87.71 kg dry assembly = 0.116976399498 kg/kg. Material input. Evangelisti et al. (2017), supplementary Hydrogen tank (Scenario S16). Preserve existing supplier proxy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A57" t="s">
         <v>25</v>
       </c>
-      <c r="B57">
-        <v>8.9411765000000004E-2</v>
+      <c r="B57" t="n">
+        <v>0.1213088587390263</v>
       </c>
       <c r="C57" t="s">
         <v>418</v>
@@ -2842,13 +2885,18 @@
       <c r="I57" t="s">
         <v>487</v>
       </c>
-    </row>
-    <row r="58" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J57" t="inlineStr">
+        <is>
+          <t>(10.64) kg / 87.71 kg dry assembly = 0.121308858739 kg/kg. Material input. Evangelisti et al. (2017), supplementary Hydrogen tank (Scenario S16). Preserve existing supplier proxy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A58" t="s">
         <v>14</v>
       </c>
-      <c r="B58">
-        <v>0.249327731</v>
+      <c r="B58" t="n">
+        <v>0.3382738570288451</v>
       </c>
       <c r="C58" t="s">
         <v>418</v>
@@ -2868,13 +2916,18 @@
       <c r="I58" t="s">
         <v>488</v>
       </c>
-    </row>
-    <row r="59" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J58" t="inlineStr">
+        <is>
+          <t>(29.67) kg / 87.71 kg dry assembly = 0.338273857029 kg/kg. Material input. Evangelisti et al. (2017), supplementary Hydrogen tank (Scenario S16). Preserve existing supplier proxy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="59" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A59" t="s">
         <v>19</v>
       </c>
-      <c r="B59">
-        <v>0.166218487</v>
+      <c r="B59" t="n">
+        <v>0.2255159046858967</v>
       </c>
       <c r="C59" t="s">
         <v>418</v>
@@ -2894,13 +2947,18 @@
       <c r="I59" t="s">
         <v>487</v>
       </c>
-    </row>
-    <row r="60" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J59" t="inlineStr">
+        <is>
+          <t>(19.78) kg / 87.71 kg dry assembly = 0.225515904686 kg/kg. Material input. Evangelisti et al. (2017), supplementary Hydrogen tank (Scenario S16). Preserve existing supplier proxy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="60" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A60" t="s">
         <v>26</v>
       </c>
-      <c r="B60">
-        <v>5.9579831999999999E-2</v>
+      <c r="B60" t="n">
+        <v>0.08083456846425721</v>
       </c>
       <c r="C60" t="s">
         <v>418</v>
@@ -2920,13 +2978,18 @@
       <c r="I60" t="s">
         <v>487</v>
       </c>
-    </row>
-    <row r="61" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J60" t="inlineStr">
+        <is>
+          <t>(7.09) kg / 87.71 kg dry assembly = 0.0808345684643 kg/kg. Material input. Evangelisti et al. (2017), supplementary Hydrogen tank (Scenario S16). Preserve existing supplier proxy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A61" t="s">
         <v>27</v>
       </c>
-      <c r="B61">
-        <v>4.7058823999999999E-2</v>
+      <c r="B61" t="n">
+        <v>0.06384676775738228</v>
       </c>
       <c r="C61" t="s">
         <v>418</v>
@@ -2945,13 +3008,18 @@
       </c>
       <c r="I61" t="s">
         <v>488</v>
+      </c>
+      <c r="J61" t="inlineStr">
+        <is>
+          <t>(5.6) kg / 87.71 kg dry assembly = 0.0638467677574 kg/kg. Material input. Evangelisti et al. (2017), supplementary Hydrogen tank (Scenario S16). Preserve existing supplier proxy.</t>
+        </is>
       </c>
     </row>
     <row r="62" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A62" t="s">
         <v>28</v>
       </c>
-      <c r="B62">
+      <c r="B62" t="n">
         <v>1</v>
       </c>
       <c r="C62" t="s">
@@ -2973,12 +3041,12 @@
         <v>488</v>
       </c>
     </row>
-    <row r="63" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="63" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A63" t="s">
         <v>29</v>
       </c>
-      <c r="B63">
-        <v>3.9243697000000001E-2</v>
+      <c r="B63" t="n">
+        <v>0.05324364382624559</v>
       </c>
       <c r="C63" t="s">
         <v>418</v>
@@ -2997,29 +3065,38 @@
       </c>
       <c r="I63" t="s">
         <v>487</v>
+      </c>
+      <c r="J63" t="inlineStr">
+        <is>
+          <t>(4.67) kg / 87.71 kg dry assembly = 0.0532436438262 kg/kg. Material input. Evangelisti et al. (2017), supplementary Hydrogen tank (Scenario S16). Preserve existing supplier proxy.</t>
+        </is>
       </c>
     </row>
     <row r="65" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A65" s="5" t="s">
         <v>1</v>
       </c>
-      <c r="B65" s="5" t="s">
-        <v>30</v>
+      <c r="B65" s="5" t="inlineStr">
+        <is>
+          <t>Fuel tank, compressed hydrogen gas, 700bar, with aluminium liner</t>
+        </is>
       </c>
     </row>
     <row r="66" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A66" t="s">
         <v>2</v>
       </c>
-      <c r="B66" t="s">
-        <v>281</v>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>RER</t>
+        </is>
       </c>
     </row>
     <row r="67" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A67" t="s">
         <v>3</v>
       </c>
-      <c r="B67">
+      <c r="B67" t="n">
         <v>1</v>
       </c>
     </row>
@@ -3027,48 +3104,60 @@
       <c r="A68" t="s">
         <v>4</v>
       </c>
-      <c r="B68" t="s">
-        <v>291</v>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>Hydrogen tank</t>
+        </is>
       </c>
     </row>
     <row r="69" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A69" t="s">
         <v>5</v>
       </c>
-      <c r="B69" t="s">
-        <v>283</v>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>process</t>
+        </is>
       </c>
     </row>
     <row r="70" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A70" t="s">
         <v>6</v>
       </c>
-      <c r="B70" t="s">
-        <v>284</v>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>kilogram</t>
+        </is>
       </c>
     </row>
     <row r="71" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A71" t="s">
         <v>7</v>
       </c>
-      <c r="B71" t="s">
-        <v>285</v>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>None</t>
+        </is>
       </c>
     </row>
     <row r="72" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A72" t="s">
         <v>8</v>
       </c>
-      <c r="B72" t="s">
-        <v>292</v>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>Evangelisti et al. 2017, doi: 10.1016/j.jclepro.2016.11.159</t>
+        </is>
       </c>
     </row>
     <row r="73" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A73" t="s">
         <v>9</v>
       </c>
-      <c r="B73" t="s">
-        <v>294</v>
+      <c r="B73" t="inlineStr">
+        <is>
+          <t>700-bar hydrogen tank with aluminium (Type III) liner. Reference output: 1 kg dry tank assembly including tank balance of plant, excluding stored hydrogen. Source listed dry materials total 113.169 kg per assembly.</t>
+        </is>
       </c>
     </row>
     <row r="74" spans="1:9" x14ac:dyDescent="0.2">
@@ -3080,18 +3169,25 @@
       <c r="A75" t="s">
         <v>11</v>
       </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>Dry-mass correction, 2026-10-10. Evangelisti et al. (2017), doi:10.1016/j.jclepro.2016.11.159, supplementary Hydrogen tank (Scenario S17). Supplement: https://ars.els-cdn.com/content/image/1-s2.0-S0959652616320212-mmc1.docx. SHA256: ca9470c504f61ef58e2e5cc3cad8c06d6cecf17073074ac2ce19dca3678ac49d. Normalize all listed material and processing quantities by 113.169 kg of listed dry materials, not the legacy 93 kg denominator. The main text, scenario labels and supplementary output masses are inconsistent. The difference between nominal output and listed material mass is approximately stored hydrogen, but this interpretation is not explicit in the paper. Dry mass is an explicit modelling boundary, not an assumed missing material. Processing services do not add material mass. Preserve published material ratios and existing supplier proxies, including AlLi for aluminium; these are not validated as current vehicle specifications. Electricity is published in MJ: divide by 3.6 to obtain kWh.</t>
+        </is>
+      </c>
     </row>
     <row r="76" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A76" s="5" t="s">
         <v>12</v>
       </c>
     </row>
-    <row r="77" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="77" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A77" s="5" t="s">
         <v>13</v>
       </c>
-      <c r="B77" s="5" t="s">
-        <v>288</v>
+      <c r="B77" s="5" t="inlineStr">
+        <is>
+          <t>amount</t>
+        </is>
       </c>
       <c r="C77" s="5" t="s">
         <v>417</v>
@@ -3114,13 +3210,18 @@
       <c r="I77" s="5" t="s">
         <v>486</v>
       </c>
-    </row>
-    <row r="78" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J77" t="inlineStr">
+        <is>
+          <t>comment</t>
+        </is>
+      </c>
+    </row>
+    <row r="78" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A78" t="s">
         <v>15</v>
       </c>
-      <c r="B78">
-        <v>0.17658064500000001</v>
+      <c r="B78" t="n">
+        <v>0.04030844724851034</v>
       </c>
       <c r="C78" t="s">
         <v>418</v>
@@ -3140,13 +3241,18 @@
       <c r="I78" t="s">
         <v>544</v>
       </c>
-    </row>
-    <row r="79" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J78" t="inlineStr">
+        <is>
+          <t>16.422 MJ / 3.6 MJ/kWh / 113.169 kg dry assembly = 0.0403084472485 kWh/kg. Evangelisti et al. (2017), supplementary Hydrogen tank (Scenario S17). Preserve existing supplier proxy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="79" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A79" t="s">
         <v>21</v>
       </c>
-      <c r="B79">
-        <v>0.11388172000000001</v>
+      <c r="B79" t="n">
+        <v>0.0935856992639327</v>
       </c>
       <c r="C79" t="s">
         <v>418</v>
@@ -3166,13 +3272,18 @@
       <c r="I79" t="s">
         <v>487</v>
       </c>
-    </row>
-    <row r="80" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J79" t="inlineStr">
+        <is>
+          <t>(10.591) kg / 113.169 kg dry assembly = 0.0935856992639 kg/kg. Processing service; excluded from material mass balance. Evangelisti et al. (2017), supplementary Hydrogen tank (Scenario S17). Preserve existing supplier proxy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="80" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A80" t="s">
         <v>25</v>
       </c>
-      <c r="B80">
-        <v>0.11388172000000001</v>
+      <c r="B80" t="n">
+        <v>0.0935856992639327</v>
       </c>
       <c r="C80" t="s">
         <v>418</v>
@@ -3192,13 +3303,18 @@
       <c r="I80" t="s">
         <v>487</v>
       </c>
-    </row>
-    <row r="81" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J80" t="inlineStr">
+        <is>
+          <t>(10.591) kg / 113.169 kg dry assembly = 0.0935856992639 kg/kg. Material input. Evangelisti et al. (2017), supplementary Hydrogen tank (Scenario S17). Preserve existing supplier proxy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="81" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A81" t="s">
         <v>14</v>
       </c>
-      <c r="B81">
-        <v>0.31989247300000001</v>
+      <c r="B81" t="n">
+        <v>0.2628811777076762</v>
       </c>
       <c r="C81" t="s">
         <v>418</v>
@@ -3218,13 +3334,18 @@
       <c r="I81" t="s">
         <v>488</v>
       </c>
-    </row>
-    <row r="82" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J81" t="inlineStr">
+        <is>
+          <t>(29.75) kg / 113.169 kg dry assembly = 0.262881177708 kg/kg. Material input. Evangelisti et al. (2017), supplementary Hydrogen tank (Scenario S17). Preserve existing supplier proxy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="82" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A82" t="s">
         <v>19</v>
       </c>
-      <c r="B82">
-        <v>0.21368817200000001</v>
+      <c r="B82" t="n">
+        <v>0.1756046267087277</v>
       </c>
       <c r="C82" t="s">
         <v>418</v>
@@ -3243,13 +3364,18 @@
       </c>
       <c r="I82" t="s">
         <v>487</v>
+      </c>
+      <c r="J82" t="inlineStr">
+        <is>
+          <t>(19.873) kg / 113.169 kg dry assembly = 0.175604626709 kg/kg. Material input. Evangelisti et al. (2017), supplementary Hydrogen tank (Scenario S17). Preserve existing supplier proxy.</t>
+        </is>
       </c>
     </row>
     <row r="83" spans="1:9" x14ac:dyDescent="0.2">
       <c r="A83" t="s">
         <v>30</v>
       </c>
-      <c r="B83">
+      <c r="B83" t="n">
         <v>1</v>
       </c>
       <c r="C83" t="s">
@@ -3271,12 +3397,12 @@
         <v>488</v>
       </c>
     </row>
-    <row r="84" spans="1:9" x14ac:dyDescent="0.2">
+    <row r="84" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A84" t="s">
         <v>31</v>
       </c>
-      <c r="B84">
-        <v>0.38387096799999998</v>
+      <c r="B84" t="n">
+        <v>0.3154574132492114</v>
       </c>
       <c r="C84" t="s">
         <v>418</v>
@@ -3296,13 +3422,18 @@
       <c r="I84" t="s">
         <v>487</v>
       </c>
-    </row>
-    <row r="85" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J84" t="inlineStr">
+        <is>
+          <t>(35.7) kg / 113.169 kg dry assembly = 0.315457413249 kg/kg. Processing service; excluded from material mass balance. Evangelisti et al. (2017), supplementary Hydrogen tank (Scenario S17). Preserve existing supplier proxy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="85" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A85" t="s">
         <v>26</v>
       </c>
-      <c r="B85">
-        <v>0.45936559100000002</v>
+      <c r="B85" t="n">
+        <v>0.377497371188223</v>
       </c>
       <c r="C85" t="s">
         <v>418</v>
@@ -3322,13 +3453,18 @@
       <c r="I85" t="s">
         <v>487</v>
       </c>
-    </row>
-    <row r="86" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J85" t="inlineStr">
+        <is>
+          <t>(35.7 + 7.021) kg / 113.169 kg dry assembly = 0.377497371188 kg/kg. Material input. Evangelisti et al. (2017), supplementary Hydrogen tank (Scenario S17). Preserve existing supplier proxy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="86" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A86" t="s">
         <v>27</v>
       </c>
-      <c r="B86">
-        <v>6.0139785000000001E-2</v>
+      <c r="B86" t="n">
+        <v>0.04942166140904311</v>
       </c>
       <c r="C86" t="s">
         <v>418</v>
@@ -3348,13 +3484,18 @@
       <c r="I86" t="s">
         <v>488</v>
       </c>
-    </row>
-    <row r="87" spans="1:9" x14ac:dyDescent="0.2">
+      <c r="J86" t="inlineStr">
+        <is>
+          <t>(5.593) kg / 113.169 kg dry assembly = 0.049421661409 kg/kg. Material input. Evangelisti et al. (2017), supplementary Hydrogen tank (Scenario S17). Preserve existing supplier proxy.</t>
+        </is>
+      </c>
+    </row>
+    <row r="87" spans="1:10" x14ac:dyDescent="0.2">
       <c r="A87" t="s">
         <v>29</v>
       </c>
-      <c r="B87">
-        <v>4.9903226000000002E-2</v>
+      <c r="B87" t="n">
+        <v>0.04100946372239748</v>
       </c>
       <c r="C87" t="s">
         <v>418</v>
@@ -3373,6 +3514,11 @@
       </c>
       <c r="I87" t="s">
         <v>487</v>
+      </c>
+      <c r="J87" t="inlineStr">
+        <is>
+          <t>(4.641) kg / 113.169 kg dry assembly = 0.0410094637224 kg/kg. Material input. Evangelisti et al. (2017), supplementary Hydrogen tank (Scenario S17). Preserve existing supplier proxy.</t>
+        </is>
       </c>
     </row>
     <row r="89" spans="1:9" x14ac:dyDescent="0.2">

</xml_diff>